<commit_message>
update oferty a w arkuszu
</commit_message>
<xml_diff>
--- a/docs/pliki/arkusz-oferty-1a.xlsx
+++ b/docs/pliki/arkusz-oferty-1a.xlsx
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00&quot; zł&quot;"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,6 +61,17 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="FF0000FF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF1F4E9A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1F4E9A"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -113,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -134,6 +145,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -573,10 +588,10 @@
           <t>l</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="14" t="n">
         <v>4.59</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="9" t="n"/>
@@ -598,10 +613,10 @@
           <t>l</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="14" t="n">
         <v>2.19</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="15" t="n">
         <v>0.3</v>
       </c>
       <c r="E6" s="9" t="n"/>
@@ -623,10 +638,10 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="14" t="n">
         <v>4.29</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="15" t="n">
         <v>0.5</v>
       </c>
       <c r="E7" s="9" t="n"/>
@@ -648,10 +663,10 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="14" t="n">
         <v>7.99</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="9" t="n"/>
@@ -673,10 +688,10 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="14" t="n">
         <v>39.99</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="15" t="n">
         <v>2.6</v>
       </c>
       <c r="E9" s="9" t="n"/>
@@ -698,10 +713,10 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="14" t="n">
         <v>71.98999999999999</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="15" t="n">
         <v>4.5</v>
       </c>
       <c r="E10" s="9" t="n"/>
@@ -723,14 +738,19 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="14" t="n">
         <v>8.49</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="15" t="n">
         <v>0.15</v>
       </c>
       <c r="E11" s="9" t="n"/>
       <c r="F11" s="9" t="n"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Niebieskie liczby to dane — wolno je zmieniać, formuły przeliczą się same.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -743,10 +763,10 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="14" t="n">
         <v>19.99</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="15" t="n">
         <v>0.4</v>
       </c>
       <c r="E12" s="9" t="n"/>
@@ -763,7 +783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -788,7 +808,7 @@
           <t>Okres (miesiące)</t>
         </is>
       </c>
-      <c r="B2" s="10" t="n">
+      <c r="B2" s="16" t="n">
         <v>24</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -845,13 +865,13 @@
           <t>sam telefon, bez dodatków</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="14" t="n">
         <v>79</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="14" t="n">
         <v>49</v>
       </c>
       <c r="F5" s="9" t="n"/>
@@ -872,13 +892,13 @@
           <t>telefon i etui</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="14" t="n">
         <v>299</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="14" t="n">
         <v>59</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="9" t="n"/>
@@ -899,13 +919,13 @@
           <t>telefon, etui, ubezpieczenie</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="14" t="n">
         <v>599</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="14" t="n">
         <v>45</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="9" t="n"/>
@@ -975,6 +995,13 @@
       <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Ceny są przykładowe, przygotowane na potrzeby ćwiczenia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Niebieskie liczby to dane — wolno je zmieniać, formuły przeliczą się same.</t>
         </is>
       </c>
     </row>
@@ -1086,13 +1113,13 @@
           <t>szt</t>
         </is>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C5" s="15" t="n">
         <v>24</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="14" t="n">
         <v>1.99</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="14" t="n">
         <v>1.69</v>
       </c>
       <c r="H5" s="6" t="inlineStr">
@@ -1117,13 +1144,13 @@
           <t>szt</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="14" t="n">
         <v>3.99</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="14" t="n">
         <v>4.29</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -1143,13 +1170,13 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="C7" s="15" t="n">
         <v>1.2</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="14" t="n">
         <v>34.9</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="14" t="n">
         <v>28.9</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -1169,13 +1196,13 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="15" t="n">
         <v>1.5</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="14" t="n">
         <v>29.9</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="14" t="n">
         <v>32.9</v>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
@@ -1191,13 +1218,13 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="C9" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="14" t="n">
         <v>7.49</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="14" t="n">
         <v>7.99</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1217,13 +1244,13 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="14" t="n">
         <v>3.49</v>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="E10" s="14" t="n">
         <v>3.99</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1243,13 +1270,13 @@
           <t>szt</t>
         </is>
       </c>
-      <c r="C11" s="8" t="n">
+      <c r="C11" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="14" t="n">
         <v>4.59</v>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="E11" s="14" t="n">
         <v>4.29</v>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1269,13 +1296,13 @@
           <t>szt</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="D12" s="14" t="n">
         <v>5.99</v>
       </c>
-      <c r="E12" s="7" t="n">
+      <c r="E12" s="14" t="n">
         <v>6.49</v>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1299,6 +1326,11 @@
       </c>
       <c r="D14" s="9" t="n"/>
       <c r="E14" s="9" t="n"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Niebieskie liczby to dane — wolno je zmieniać, formuły przeliczą się same.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1306,10 +1338,10 @@
           <t>Koszt dojazdu</t>
         </is>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E15" s="17" t="n">
         <v>18</v>
       </c>
     </row>

</xml_diff>